<commit_message>
AK47DX V14.1 FIX4 template Tempo obiettivo
</commit_message>
<xml_diff>
--- a/public/templates/TEMPLATE_IMPORT_RISULTATI_CODM_CLAN_MANAGER_V12_1_FOTO_PROFILI.xlsx
+++ b/public/templates/TEMPLATE_IMPORT_RISULTATI_CODM_CLAN_MANAGER_V12_1_FOTO_PROFILI.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IMPORT_PARTITE" sheetId="1" r:id="Ra37e91ddc09a425f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ESEMPIO_COMPILATO" sheetId="2" r:id="Rc0515ba6492848ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LISTE" sheetId="3" r:id="R55c6c5cf4e3f414b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ISTRUZIONI" sheetId="4" r:id="R0f3d6ffef8ad48a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IMPORT_PARTITE" sheetId="1" r:id="Rc68e4c4c8bd2437c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ESEMPIO_COMPILATO" sheetId="2" r:id="R4892651c4bac41d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LISTE" sheetId="3" r:id="Rb390132f801f4cdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ISTRUZIONI" sheetId="4" r:id="Rfb93276445384688"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,7 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="4">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -38,8 +38,19 @@
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF155E4B"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1E2C36"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -61,6 +72,26 @@
         <x:fgColor rgb="FFE5E7EB"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF242B35"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF177E65"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE5F4EE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE6EDF1"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -69,7 +100,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="32">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -112,6 +143,34 @@
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -228,9 +287,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -334,108 +393,112 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="17" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="17" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="20" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="26" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="18" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="18" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="18" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="18" hidden="0" customWidth="1"/>
-    <x:col min="22" max="22" width="18" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="32" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="34" hidden="0" customWidth="1"/>
-    <x:col min="25" max="25" width="40" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="20" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="20" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="20" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="12" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="12" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="12" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="12" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="22" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="22" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="22" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="22" t="str">
         <x:v>ID_PARTITA</x:v>
       </x:c>
-      <x:c r="B1" s="5" t="str">
+      <x:c r="B1" s="22" t="str">
         <x:v>DATA</x:v>
       </x:c>
-      <x:c r="C1" s="5" t="str">
+      <x:c r="C1" s="22" t="str">
         <x:v>ORA</x:v>
       </x:c>
-      <x:c r="D1" s="5" t="str">
+      <x:c r="D1" s="22" t="str">
         <x:v>TIPO_PARTITA</x:v>
       </x:c>
-      <x:c r="E1" s="5" t="str">
+      <x:c r="E1" s="22" t="str">
         <x:v>MODALITA_CODM</x:v>
       </x:c>
-      <x:c r="F1" s="5" t="str">
+      <x:c r="F1" s="22" t="str">
         <x:v>MAPPA_CODM</x:v>
       </x:c>
-      <x:c r="G1" s="5" t="str">
+      <x:c r="G1" s="22" t="str">
         <x:v>TEAM_NOSTRO</x:v>
       </x:c>
-      <x:c r="H1" s="5" t="str">
+      <x:c r="H1" s="22" t="str">
         <x:v>TEAM_BLU</x:v>
       </x:c>
-      <x:c r="I1" s="5" t="str">
+      <x:c r="I1" s="22" t="str">
         <x:v>TEAM_ROSSO</x:v>
       </x:c>
-      <x:c r="J1" s="5" t="str">
+      <x:c r="J1" s="22" t="str">
         <x:v>RISULTATO_BLU</x:v>
       </x:c>
-      <x:c r="K1" s="5" t="str">
+      <x:c r="K1" s="22" t="str">
         <x:v>RISULTATO_ROSSO</x:v>
       </x:c>
-      <x:c r="L1" s="5" t="str">
+      <x:c r="L1" s="22" t="str">
         <x:v>RISULTATO_NOSTRO</x:v>
       </x:c>
-      <x:c r="M1" s="5" t="str">
+      <x:c r="M1" s="22" t="str">
         <x:v>RISULTATO_AVVERSARIO</x:v>
       </x:c>
-      <x:c r="N1" s="5" t="str">
+      <x:c r="N1" s="22" t="str">
         <x:v>ESITO_NOSTRO</x:v>
       </x:c>
-      <x:c r="O1" s="5" t="str">
+      <x:c r="O1" s="22" t="str">
         <x:v>GIOCATORE</x:v>
       </x:c>
-      <x:c r="P1" s="5" t="str">
+      <x:c r="P1" s="22" t="str">
         <x:v>GIOCATORE_EMAIL</x:v>
       </x:c>
-      <x:c r="Q1" s="5" t="str">
+      <x:c r="Q1" s="22" t="str">
         <x:v>UID_CODM</x:v>
       </x:c>
-      <x:c r="R1" s="5" t="str">
+      <x:c r="R1" s="22" t="str">
         <x:v>TEAM_GIOCATORE</x:v>
       </x:c>
-      <x:c r="S1" s="5" t="str">
+      <x:c r="S1" s="22" t="str">
         <x:v>KILL</x:v>
       </x:c>
-      <x:c r="T1" s="5" t="str">
+      <x:c r="T1" s="22" t="str">
         <x:v>DEATH</x:v>
       </x:c>
-      <x:c r="U1" s="5" t="str">
+      <x:c r="U1" s="22" t="str">
         <x:v>ASSIST</x:v>
       </x:c>
-      <x:c r="V1" s="5" t="str">
+      <x:c r="V1" s="22" t="str">
         <x:v>MVP</x:v>
       </x:c>
-      <x:c r="W1" s="5" t="str">
+      <x:c r="W1" s="22" t="str">
         <x:v>FOTO_FILE</x:v>
       </x:c>
-      <x:c r="X1" s="5" t="str">
+      <x:c r="X1" s="22" t="str">
         <x:v>FOTO_URL</x:v>
       </x:c>
-      <x:c r="Y1" s="5" t="str">
+      <x:c r="Y1" s="22" t="str">
         <x:v>NOTE</x:v>
+      </x:c>
+      <x:c r="Z1" s="25" t="str">
+        <x:v>TEMPO_OBIETTIVO</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -1814,7 +1877,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03d6ffadd3334532"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b578b6c3f21416f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1823,116 +1886,120 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="17" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="17" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="20" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="26" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="18" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="18" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="18" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="18" hidden="0" customWidth="1"/>
-    <x:col min="22" max="22" width="18" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="32" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="34" hidden="0" customWidth="1"/>
-    <x:col min="25" max="25" width="40" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="20" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="20" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="20" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="12" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="12" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="12" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="12" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="22" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="22" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="22" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="22" t="str">
         <x:v>ID_PARTITA</x:v>
       </x:c>
-      <x:c r="B1" s="5" t="str">
+      <x:c r="B1" s="22" t="str">
         <x:v>DATA</x:v>
       </x:c>
-      <x:c r="C1" s="5" t="str">
+      <x:c r="C1" s="22" t="str">
         <x:v>ORA</x:v>
       </x:c>
-      <x:c r="D1" s="5" t="str">
+      <x:c r="D1" s="22" t="str">
         <x:v>TIPO_PARTITA</x:v>
       </x:c>
-      <x:c r="E1" s="5" t="str">
+      <x:c r="E1" s="22" t="str">
         <x:v>MODALITA_CODM</x:v>
       </x:c>
-      <x:c r="F1" s="5" t="str">
+      <x:c r="F1" s="22" t="str">
         <x:v>MAPPA_CODM</x:v>
       </x:c>
-      <x:c r="G1" s="5" t="str">
+      <x:c r="G1" s="22" t="str">
         <x:v>TEAM_NOSTRO</x:v>
       </x:c>
-      <x:c r="H1" s="5" t="str">
+      <x:c r="H1" s="22" t="str">
         <x:v>TEAM_BLU</x:v>
       </x:c>
-      <x:c r="I1" s="5" t="str">
+      <x:c r="I1" s="22" t="str">
         <x:v>TEAM_ROSSO</x:v>
       </x:c>
-      <x:c r="J1" s="5" t="str">
+      <x:c r="J1" s="22" t="str">
         <x:v>RISULTATO_BLU</x:v>
       </x:c>
-      <x:c r="K1" s="5" t="str">
+      <x:c r="K1" s="22" t="str">
         <x:v>RISULTATO_ROSSO</x:v>
       </x:c>
-      <x:c r="L1" s="5" t="str">
+      <x:c r="L1" s="22" t="str">
         <x:v>RISULTATO_NOSTRO</x:v>
       </x:c>
-      <x:c r="M1" s="5" t="str">
+      <x:c r="M1" s="22" t="str">
         <x:v>RISULTATO_AVVERSARIO</x:v>
       </x:c>
-      <x:c r="N1" s="5" t="str">
+      <x:c r="N1" s="22" t="str">
         <x:v>ESITO_NOSTRO</x:v>
       </x:c>
-      <x:c r="O1" s="5" t="str">
+      <x:c r="O1" s="22" t="str">
         <x:v>GIOCATORE</x:v>
       </x:c>
-      <x:c r="P1" s="5" t="str">
+      <x:c r="P1" s="22" t="str">
         <x:v>GIOCATORE_EMAIL</x:v>
       </x:c>
-      <x:c r="Q1" s="5" t="str">
+      <x:c r="Q1" s="22" t="str">
         <x:v>UID_CODM</x:v>
       </x:c>
-      <x:c r="R1" s="5" t="str">
+      <x:c r="R1" s="22" t="str">
         <x:v>TEAM_GIOCATORE</x:v>
       </x:c>
-      <x:c r="S1" s="5" t="str">
+      <x:c r="S1" s="22" t="str">
         <x:v>KILL</x:v>
       </x:c>
-      <x:c r="T1" s="5" t="str">
+      <x:c r="T1" s="22" t="str">
         <x:v>DEATH</x:v>
       </x:c>
-      <x:c r="U1" s="5" t="str">
+      <x:c r="U1" s="22" t="str">
         <x:v>ASSIST</x:v>
       </x:c>
-      <x:c r="V1" s="5" t="str">
+      <x:c r="V1" s="22" t="str">
         <x:v>MVP</x:v>
       </x:c>
-      <x:c r="W1" s="5" t="str">
+      <x:c r="W1" s="22" t="str">
         <x:v>FOTO_FILE</x:v>
       </x:c>
-      <x:c r="X1" s="5" t="str">
+      <x:c r="X1" s="22" t="str">
         <x:v>FOTO_URL</x:v>
       </x:c>
-      <x:c r="Y1" s="5" t="str">
+      <x:c r="Y1" s="22" t="str">
         <x:v>NOTE</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2">
+      <x:c r="Z1" s="25" t="str">
+        <x:v>TEMPO_OBIETTIVO</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" t="str">
-        <x:v>CED_20260708_001</x:v>
+        <x:v>DEMO_POST_001</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>2026-07-08</x:v>
+        <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C2" t="str">
         <x:v>21:00</x:v>
@@ -1944,7 +2011,7 @@
         <x:v>POSTAZIONE</x:v>
       </x:c>
       <x:c r="F2" t="str">
-        <x:v>Standoff</x:v>
+        <x:v>Raid</x:v>
       </x:c>
       <x:c r="G2" t="str">
         <x:v>BLU</x:v>
@@ -1953,59 +2020,60 @@
         <x:v>AK47DX</x:v>
       </x:c>
       <x:c r="I2" t="str">
-        <x:v>AVVERSARI</x:v>
+        <x:v>CLAN ESEMPIO</x:v>
       </x:c>
       <x:c r="J2" t="n">
-        <x:v>6</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K2" t="n">
-        <x:v>0</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="L2" t="n">
-        <x:v>6</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="M2" t="n">
-        <x:v>0</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="N2" t="str">
         <x:v>WIN</x:v>
       </x:c>
       <x:c r="O2" t="str">
-        <x:v>MIRZA</x:v>
-      </x:c>
-      <x:c r="P2" t="str">
-        <x:v>hasnaiiin@gmail.com</x:v>
-      </x:c>
+        <x:v>Giocatore 1</x:v>
+      </x:c>
+      <x:c r="P2" t="str"/>
       <x:c r="Q2" t="str"/>
       <x:c r="R2" t="str">
         <x:v>NOSTRO</x:v>
       </x:c>
       <x:c r="S2" t="n">
-        <x:v>18</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="T2" t="n">
-        <x:v>7</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="U2" t="n">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="V2" t="str">
         <x:v>SI</x:v>
       </x:c>
       <x:c r="W2" t="str">
-        <x:v>CED_20260708_001_scoreboard.jpg</x:v>
+        <x:v>DEMO_POST_001_prova.jpg</x:v>
       </x:c>
       <x:c r="X2" t="str"/>
       <x:c r="Y2" t="str">
-        <x:v>Esempio: foto da allegare subito o dopo</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z2" s="27" t="str">
+        <x:v>01:35</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" t="str">
-        <x:v>CED_20260708_001</x:v>
+        <x:v>DEMO_POST_001</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>2026-07-08</x:v>
+        <x:v>2026-10-01</x:v>
       </x:c>
       <x:c r="C3" t="str">
         <x:v>21:00</x:v>
@@ -2017,7 +2085,7 @@
         <x:v>POSTAZIONE</x:v>
       </x:c>
       <x:c r="F3" t="str">
-        <x:v>Standoff</x:v>
+        <x:v>Raid</x:v>
       </x:c>
       <x:c r="G3" t="str">
         <x:v>BLU</x:v>
@@ -2026,25 +2094,25 @@
         <x:v>AK47DX</x:v>
       </x:c>
       <x:c r="I3" t="str">
-        <x:v>AVVERSARI</x:v>
+        <x:v>CLAN ESEMPIO</x:v>
       </x:c>
       <x:c r="J3" t="n">
-        <x:v>6</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K3" t="n">
-        <x:v>0</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="L3" t="n">
-        <x:v>6</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="M3" t="n">
-        <x:v>0</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="N3" t="str">
         <x:v>WIN</x:v>
       </x:c>
       <x:c r="O3" t="str">
-        <x:v>Player2</x:v>
+        <x:v>Giocatore 2</x:v>
       </x:c>
       <x:c r="P3" t="str"/>
       <x:c r="Q3" t="str"/>
@@ -2052,29 +2120,1350 @@
         <x:v>NOSTRO</x:v>
       </x:c>
       <x:c r="S3" t="n">
-        <x:v>12</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="T3" t="n">
-        <x:v>9</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="U3" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="V3" t="str">
         <x:v>NO</x:v>
       </x:c>
       <x:c r="W3" t="str">
-        <x:v>CED_20260708_001_scoreboard.jpg</x:v>
+        <x:v>DEMO_POST_001_prova.jpg</x:v>
       </x:c>
       <x:c r="X3" t="str"/>
       <x:c r="Y3" t="str">
-        <x:v>Stessa partita, seconda riga player</x:v>
-      </x:c>
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z3" s="27" t="str">
+        <x:v>00:58</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" t="str">
+        <x:v>DEMO_POST_001</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>2026-10-01</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>21:00</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>POSTAZIONE</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>Raid</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J4" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="K4" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="L4" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="M4" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="N4" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O4" t="str">
+        <x:v>Giocatore 3</x:v>
+      </x:c>
+      <x:c r="P4" t="str"/>
+      <x:c r="Q4" t="str"/>
+      <x:c r="R4" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S4" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="T4" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="U4" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="V4" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="W4" t="str">
+        <x:v>DEMO_POST_001_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X4" t="str"/>
+      <x:c r="Y4" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z4" s="27" t="str">
+        <x:v>01:12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" t="str">
+        <x:v>DEMO_POST_001</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>2026-10-01</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>21:00</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>POSTAZIONE</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>Raid</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J5" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="K5" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="L5" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="M5" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="N5" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O5" t="str">
+        <x:v>Giocatore 4</x:v>
+      </x:c>
+      <x:c r="P5" t="str"/>
+      <x:c r="Q5" t="str"/>
+      <x:c r="R5" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S5" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="T5" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="U5" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="V5" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="W5" t="str">
+        <x:v>DEMO_POST_001_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X5" t="str"/>
+      <x:c r="Y5" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z5" s="27" t="str">
+        <x:v>00:42</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" t="str">
+        <x:v>DEMO_POST_001</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>2026-10-01</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>21:00</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>POSTAZIONE</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>Raid</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J6" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="K6" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="L6" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="M6" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="N6" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O6" t="str">
+        <x:v>Giocatore 5</x:v>
+      </x:c>
+      <x:c r="P6" t="str"/>
+      <x:c r="Q6" t="str"/>
+      <x:c r="R6" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S6" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="T6" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="U6" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="V6" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="W6" t="str">
+        <x:v>DEMO_POST_001_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X6" t="str"/>
+      <x:c r="Y6" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z6" s="27" t="str">
+        <x:v>02:05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="A7" t="str">
+        <x:v>DEMO_DOM_002</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>2026-10-02</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>21:15</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>DOMINIO</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>Standoff</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J7" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="K7" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="L7" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="M7" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="N7" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O7" t="str">
+        <x:v>Giocatore 1</x:v>
+      </x:c>
+      <x:c r="P7" t="str"/>
+      <x:c r="Q7" t="str"/>
+      <x:c r="R7" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S7" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="T7" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="U7" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="V7" t="str">
+        <x:v>SI</x:v>
+      </x:c>
+      <x:c r="W7" t="str">
+        <x:v>DEMO_DOM_002_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X7" t="str"/>
+      <x:c r="Y7" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z7" s="27" t="str">
+        <x:v>00:35</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="22" customHeight="1">
+      <x:c r="A8" t="str">
+        <x:v>DEMO_DOM_002</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>2026-10-02</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>21:15</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>DOMINIO</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>Standoff</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J8" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="K8" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="L8" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="M8" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="N8" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O8" t="str">
+        <x:v>Giocatore 2</x:v>
+      </x:c>
+      <x:c r="P8" t="str"/>
+      <x:c r="Q8" t="str"/>
+      <x:c r="R8" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S8" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="T8" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="U8" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="V8" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="W8" t="str">
+        <x:v>DEMO_DOM_002_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X8" t="str"/>
+      <x:c r="Y8" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z8" s="27" t="str">
+        <x:v>01:03</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="22" customHeight="1">
+      <x:c r="A9" t="str">
+        <x:v>DEMO_DOM_002</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>2026-10-02</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>21:15</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>DOMINIO</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>Standoff</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I9" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J9" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="K9" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="L9" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="M9" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="N9" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O9" t="str">
+        <x:v>Giocatore 3</x:v>
+      </x:c>
+      <x:c r="P9" t="str"/>
+      <x:c r="Q9" t="str"/>
+      <x:c r="R9" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S9" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="T9" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="U9" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="V9" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="W9" t="str">
+        <x:v>DEMO_DOM_002_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X9" t="str"/>
+      <x:c r="Y9" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z9" s="27" t="str">
+        <x:v>00:41</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="22" customHeight="1">
+      <x:c r="A10" t="str">
+        <x:v>DEMO_DOM_002</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>2026-10-02</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>21:15</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>DOMINIO</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>Standoff</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J10" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="K10" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="L10" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="M10" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="N10" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O10" t="str">
+        <x:v>Giocatore 4</x:v>
+      </x:c>
+      <x:c r="P10" t="str"/>
+      <x:c r="Q10" t="str"/>
+      <x:c r="R10" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S10" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="T10" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="U10" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="V10" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="W10" t="str">
+        <x:v>DEMO_DOM_002_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X10" t="str"/>
+      <x:c r="Y10" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z10" s="27" t="str">
+        <x:v>00:55</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="22" customHeight="1">
+      <x:c r="A11" t="str">
+        <x:v>DEMO_DOM_002</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>2026-10-02</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>21:15</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>DOMINIO</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>Standoff</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J11" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="K11" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="L11" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="M11" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="N11" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O11" t="str">
+        <x:v>Giocatore 5</x:v>
+      </x:c>
+      <x:c r="P11" t="str"/>
+      <x:c r="Q11" t="str"/>
+      <x:c r="R11" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S11" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="T11" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="U11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="V11" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="W11" t="str">
+        <x:v>DEMO_DOM_002_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X11" t="str"/>
+      <x:c r="Y11" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z11" s="27" t="str">
+        <x:v>00:28</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="22" customHeight="1">
+      <x:c r="A12" t="str">
+        <x:v>DEMO_CTRL_003</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>2026-10-03</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>21:30</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>CONTROLLO</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>Firing Range</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N12" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O12" t="str">
+        <x:v>Giocatore 1</x:v>
+      </x:c>
+      <x:c r="P12" t="str"/>
+      <x:c r="Q12" t="str"/>
+      <x:c r="R12" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S12" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="T12" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="U12" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="V12" t="str">
+        <x:v>SI</x:v>
+      </x:c>
+      <x:c r="W12" t="str">
+        <x:v>DEMO_CTRL_003_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X12" t="str"/>
+      <x:c r="Y12" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z12" s="27" t="str">
+        <x:v>00:44</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="22" customHeight="1">
+      <x:c r="A13" t="str">
+        <x:v>DEMO_CTRL_003</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>2026-10-03</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>21:30</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>CONTROLLO</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>Firing Range</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I13" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J13" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L13" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N13" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O13" t="str">
+        <x:v>Giocatore 2</x:v>
+      </x:c>
+      <x:c r="P13" t="str"/>
+      <x:c r="Q13" t="str"/>
+      <x:c r="R13" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S13" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="T13" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="U13" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="V13" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="W13" t="str">
+        <x:v>DEMO_CTRL_003_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X13" t="str"/>
+      <x:c r="Y13" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z13" s="27" t="str">
+        <x:v>00:51</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="22" customHeight="1">
+      <x:c r="A14" t="str">
+        <x:v>DEMO_CTRL_003</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>2026-10-03</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>21:30</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>CONTROLLO</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>Firing Range</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I14" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J14" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K14" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L14" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M14" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N14" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O14" t="str">
+        <x:v>Giocatore 3</x:v>
+      </x:c>
+      <x:c r="P14" t="str"/>
+      <x:c r="Q14" t="str"/>
+      <x:c r="R14" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S14" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="T14" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="U14" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="V14" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="W14" t="str">
+        <x:v>DEMO_CTRL_003_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X14" t="str"/>
+      <x:c r="Y14" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z14" s="27" t="str"/>
+    </x:row>
+    <x:row r="15" ht="22" customHeight="1">
+      <x:c r="A15" t="str">
+        <x:v>DEMO_CTRL_003</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>2026-10-03</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>21:30</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>CONTROLLO</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>Firing Range</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N15" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O15" t="str">
+        <x:v>Giocatore 4</x:v>
+      </x:c>
+      <x:c r="P15" t="str"/>
+      <x:c r="Q15" t="str"/>
+      <x:c r="R15" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S15" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="T15" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="U15" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="V15" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="W15" t="str">
+        <x:v>DEMO_CTRL_003_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X15" t="str"/>
+      <x:c r="Y15" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z15" s="27" t="str">
+        <x:v>00:32</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="22" customHeight="1">
+      <x:c r="A16" t="str">
+        <x:v>DEMO_CTRL_003</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>2026-10-03</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>21:30</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>CONTROLLO</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>Firing Range</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I16" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J16" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L16" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N16" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O16" t="str">
+        <x:v>Giocatore 5</x:v>
+      </x:c>
+      <x:c r="P16" t="str"/>
+      <x:c r="Q16" t="str"/>
+      <x:c r="R16" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S16" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="T16" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="U16" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="V16" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="W16" t="str">
+        <x:v>DEMO_CTRL_003_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X16" t="str"/>
+      <x:c r="Y16" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z16" s="27" t="str"/>
+    </x:row>
+    <x:row r="17" ht="22" customHeight="1">
+      <x:c r="A17" t="str">
+        <x:v>DEMO_CED_004</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>22:00</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>CED</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>Summit</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I17" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J17" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L17" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="M17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N17" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O17" t="str">
+        <x:v>Giocatore 1</x:v>
+      </x:c>
+      <x:c r="P17" t="str"/>
+      <x:c r="Q17" t="str"/>
+      <x:c r="R17" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S17" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="T17" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="U17" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="V17" t="str">
+        <x:v>SI</x:v>
+      </x:c>
+      <x:c r="W17" t="str">
+        <x:v>DEMO_CED_004_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X17" t="str"/>
+      <x:c r="Y17" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z17" s="27" t="str"/>
+    </x:row>
+    <x:row r="18" ht="22" customHeight="1">
+      <x:c r="A18" t="str">
+        <x:v>DEMO_CED_004</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>22:00</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>CED</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>Summit</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I18" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J18" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L18" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="M18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N18" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O18" t="str">
+        <x:v>Giocatore 2</x:v>
+      </x:c>
+      <x:c r="P18" t="str"/>
+      <x:c r="Q18" t="str"/>
+      <x:c r="R18" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S18" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="T18" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="U18" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="V18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="W18" t="str">
+        <x:v>DEMO_CED_004_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X18" t="str"/>
+      <x:c r="Y18" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z18" s="27" t="str"/>
+    </x:row>
+    <x:row r="19" ht="22" customHeight="1">
+      <x:c r="A19" t="str">
+        <x:v>DEMO_CED_004</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>22:00</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>CED</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>Summit</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I19" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J19" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K19" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L19" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="M19" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N19" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O19" t="str">
+        <x:v>Giocatore 3</x:v>
+      </x:c>
+      <x:c r="P19" t="str"/>
+      <x:c r="Q19" t="str"/>
+      <x:c r="R19" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S19" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="T19" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="U19" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="V19" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="W19" t="str">
+        <x:v>DEMO_CED_004_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X19" t="str"/>
+      <x:c r="Y19" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z19" s="27" t="str"/>
+    </x:row>
+    <x:row r="20" ht="22" customHeight="1">
+      <x:c r="A20" t="str">
+        <x:v>DEMO_CED_004</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>22:00</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>CED</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>Summit</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I20" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J20" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L20" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="M20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N20" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O20" t="str">
+        <x:v>Giocatore 4</x:v>
+      </x:c>
+      <x:c r="P20" t="str"/>
+      <x:c r="Q20" t="str"/>
+      <x:c r="R20" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S20" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="T20" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="U20" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="V20" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="W20" t="str">
+        <x:v>DEMO_CED_004_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X20" t="str"/>
+      <x:c r="Y20" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z20" s="27" t="str"/>
+    </x:row>
+    <x:row r="21" ht="22" customHeight="1">
+      <x:c r="A21" t="str">
+        <x:v>DEMO_CED_004</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>22:00</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>scrim</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>CED</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>Summit</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>BLU</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>AK47DX</x:v>
+      </x:c>
+      <x:c r="I21" t="str">
+        <x:v>CLAN ESEMPIO</x:v>
+      </x:c>
+      <x:c r="J21" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K21" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L21" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="M21" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N21" t="str">
+        <x:v>WIN</x:v>
+      </x:c>
+      <x:c r="O21" t="str">
+        <x:v>Giocatore 5</x:v>
+      </x:c>
+      <x:c r="P21" t="str"/>
+      <x:c r="Q21" t="str"/>
+      <x:c r="R21" t="str">
+        <x:v>NOSTRO</x:v>
+      </x:c>
+      <x:c r="S21" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="T21" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="U21" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="V21" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="W21" t="str">
+        <x:v>DEMO_CED_004_prova.jpg</x:v>
+      </x:c>
+      <x:c r="X21" t="str"/>
+      <x:c r="Y21" t="str">
+        <x:v>DATI DIMOSTRATIVI, NON IMPORTARE COME PARTITA REALE</x:v>
+      </x:c>
+      <x:c r="Z21" s="27" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf325cd4902294342"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R524759c28f40492b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2458,15 +3847,15 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="91.5" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="143.1300048828125" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="29" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="102" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="13" t="str">
-        <x:v>CLAN MANAGER V12.1 - Template import risultati Excel + foto prova + profilo reale</x:v>
-      </x:c>
-      <x:c r="B1" s="10"/>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="28" t="str">
+        <x:v>CLAN MANAGER V14.1 — Template risultati con Tempo obiettivo per giocatore</x:v>
+      </x:c>
+      <x:c r="B1" s="23"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="10" t="str"/>
@@ -2510,6 +3899,46 @@
       </x:c>
       <x:c r="B7" s="10" t="str">
         <x:v>Per caricamento SQL usare supabase/IMPORT_RISULTATI_EXCEL_STAGING_V12.sql e supabase/LOAD_RISULTATI_ESEMPIO_V12.sql come base.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="34" customHeight="1">
+      <x:c r="A8" s="31" t="str">
+        <x:v>TEMPO_OBIETTIVO</x:v>
+      </x:c>
+      <x:c r="B8" s="10" t="str">
+        <x:v>Colonna Z. Scrivi 01:35, 00:48 ecc. (mm:ss). Lascia vuoto se non disponibile. NON inserire numeri nudi come 95.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="31" t="str">
+        <x:v>Modalità</x:v>
+      </x:c>
+      <x:c r="B9" s="10" t="str">
+        <x:v>POSTAZIONE, DOMINIO, CONTROLLO e CED: il tempo si usa solo se visibile o verificato. Per CED solitamente è vuoto.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="34" customHeight="1">
+      <x:c r="A10" s="31" t="str">
+        <x:v>ISTRUZIONI IMPORT</x:v>
+      </x:c>
+      <x:c r="B10" s="10" t="str">
+        <x:v>Compila IMPORT_PARTITE (scheda vuota). ESEMPIO_COMPILATO contiene SOLTANTO dati dimostrativi: non importare l'esempio come partite vere.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="34" customHeight="1">
+      <x:c r="A11" s="31" t="str">
+        <x:v>Passi sul sito</x:v>
+      </x:c>
+      <x:c r="B11" s="10" t="str">
+        <x:v>Partite &gt; Importa partita &gt; Dati partita &gt; Importa risultato da Excel o tabella &gt; Carica Excel. Verifica Tempo obiettivo in tabella giocatori e premi Salva.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="34" customHeight="1">
+      <x:c r="A12" s="31" t="str">
+        <x:v>Prerequisito Supabase</x:v>
+      </x:c>
+      <x:c r="B12" s="10" t="str">
+        <x:v>Colonne objective_time_seconds e objective_time_text su match_scoreboard_rows e match_player_stats (migrazione V14).</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>